<commit_message>
Review log: shorten all comments to one short phrase per cell
</commit_message>
<xml_diff>
--- a/CS-Testing/06-Requirements-Review/SOW1-SOW2_Review_Log.xlsx
+++ b/CS-Testing/06-Requirements-Review/SOW1-SOW2_Review_Log.xlsx
@@ -469,17 +469,17 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -576,46 +576,38 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>• Frames 1-17 carry no tag: drop, accept or show?
-• Which rows does the CMAC cover?</t>
+          <t>Frames 1-17 have no tag: how to treat?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>• Text says 'each frame'; imager tags only frames 18+ and only selected rows.
-• Reword: 'each frame that carries a tag, over the selected rows'. Add a requirement for untagged frames.</t>
+          <t>Says 'each frame'; only frames 18+ are tagged. Reword.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>• Comparison is internal; same observable as 119710. Use the log event or a drop counter.
-• SIM needed: tester must know the session key.</t>
+          <t>Not observable alone; same as 119710.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>• Unselected rows and statistics are not authenticated.
-• No latency limit for holding a frame until verified.</t>
+          <t>Only selected rows are authenticated.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>• Merge with 119710, or split compare (119709) from reaction (119710).
-• TCR 106582 copies the text: add algorithm and input.</t>
+          <t>Merge with 119710.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106582 (ok).
-• Upstream MVC-106231 is too generic.
-• SRS 108112/108117/108122: link missing.</t>
+          <t>MVC-106582. SRS link missing.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>SIM: correct tag -&gt; frame accepted (RTP seen)
-SIM: flip 1 tag bit / truncate / wrong key / zero tag -&gt; rejected
-UART log: 'CMAC failed'</t>
+          <t>SIM sends good tag -&gt; accepted
+SIM flips 1 tag bit -&gt; rejected, log</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -647,42 +639,38 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>• PSS salt length and MGF?
-• Does KID select the scheme (SRS 108135)?</t>
+          <t>PSS salt length? Does KID select the scheme?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>• If only PSS/SHA-256 exists, drop the KID selection in the SRS; otherwise list accepted KIDs.</t>
+          <t>Define salt and MGF; align SRS on KID.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>• Partly inspection.
-• PKCS#1 v1.5 or another hash must fail; salt cases need the salt defined.</t>
+          <t>Partly inspection; salt untestable until defined.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>• Salt length, MGF and exponent are not stated.</t>
+          <t>Salt, MGF, exponent not stated.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>• Property of the 107642 verification: merge or keep as technical detail.</t>
+          <t>Merge into 107642.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>• MVC-106563 does not link back: add the link.
-• SRS 108120, 108135, 108136.</t>
+          <t>MVC-106563 not linked back.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Review: verify call = RSASSA-PSS + SHA-256
-PyRef: PSS/SHA-256 -&gt; accepted
-PKCS#1 v1.5, SHA-1, SHA-384 -&gt; rejected</t>
+          <t>Code review: PSS + SHA-256
+PyRef: v1.5 or SHA-1 signature -&gt; rejected</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -693,7 +681,7 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
     </row>
-    <row r="4" ht="66" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -714,44 +702,38 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>• Which DRBG and TRNG interface?
-• Evidence for SP 800-90A and TRNG quality (Ambarella)?</t>
+          <t>Which DRBG and TRNG? Compliance evidence?</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>• Conformity is a design property: change the method to Review.
-• Keep a test for the failure behaviour.</t>
+          <t>Change method to Review.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>• Black-box shows only uniqueness.
-• Inject a TRNG error with Lauterbach.</t>
+          <t>Black-box shows only uniqueness.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>• SP 800-90A covers the DRBG, not the entropy source (800-90B).
-• No reseed rule.</t>
+          <t>No reseed rule.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>• Same TRNG as debug requirement MVC-103050.</t>
+          <t>Same TRNG as MVC-103050.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106560.
-• SRS 108106, 108109, 23.1.1.2.</t>
+          <t>MVC-106560.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Review: DRBG type and TRNG seed call; collect evidence
-Lauterbach: force TRNG error -&gt; no key block (Saleae)
-Collect 1000 SSKs via SIM -&gt; no repeats</t>
+          <t>Review DRBG + TRNG evidence
+Lauterbach: force TRNG error -&gt; no key sent</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -783,22 +765,22 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>• How does SOW2 know the imager accepted the key block?</t>
+          <t>How does SOW2 know the key was accepted?</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>• 'Session established' is undefined; 119708, 103046, 103044 depend on it.</t>
+          <t>'Session established' is undefined.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>• Capture the write with Saleae; layout from the Samsung note.</t>
+          <t>Saleae capture; layout needed.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>• I2C CRC is ON (Volvo spec); a 256-byte block may need several writes: partial writes undefined.</t>
+          <t>Block may need several I2C writes.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -808,15 +790,13 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106578.
-• SRS 108146, 108145.</t>
+          <t>MVC-106578.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Saleae: after auth OK, write to imager key register = encrypted block, right length
-Order: auth read -&gt; verify -&gt; key write
-SIM acks -&gt; SESSION_ACTIVE; silent -&gt; not active</t>
+          <t>Saleae: key write only after auth OK
+SIM no ack -&gt; no session</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -848,44 +828,38 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>• After termination: no video, retry later, or safe state?
-• When is the next attempt allowed?</t>
+          <t>Reaction after termination: no video or safe state?</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>• A cybersecurity failure can switch off the camera image.
-• Define the reaction with FuSa.</t>
+          <t>Can switch off the camera image. Define reaction.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>• End state is observable (state, bus, stream).
-• 'No retry forever' needs a defined observation time.</t>
+          <t>End state is observable.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>• Concept says 'configured maximum', technical says a fixed three.</t>
+          <t>'Configured' vs fixed three.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>• See 103053.</t>
+          <t>See 103053.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106569.
-• SRS 108124 is similar.</t>
+          <t>MVC-106569.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>SIM never gives valid data; reset
-Saleae: no auth request or key write for 60 s
-Lauterbach: state UNAUTHENTICATED; valid-tag frames rejected
-Power cycle -&gt; new attempt</t>
+          <t>SIM never answers -&gt; Saleae: no more requests
+Lauterbach: state UNAUTHENTICATED</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -917,22 +891,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>• Reaction after termination: no video, new auth, or safe state?</t>
+          <t>Reaction after termination?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>• Define the next step and whether retries restart after a new authentication.</t>
+          <t>Define the next step.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>• End state is observable: no session, no more writes, key unused.</t>
+          <t>End state is observable.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>• The failed attempt's SSK must be erased (SRS 108149): check the buffer.</t>
+          <t>Erase the failed attempt's SSK.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -942,16 +916,13 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106581.
-• SRS 108149, 108158.</t>
+          <t>MVC-106581.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>SIM never acks the key block
-Saleae: no key writes for 60 s after last retry
-Lauterbach: state INACTIVE, key buffer zero
-Tagged frames rejected; reset -&gt; new attempt</t>
+          <t>SIM never acks -&gt; no more key writes
+Lauterbach: key buffer zero</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -962,7 +933,7 @@
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
     </row>
-    <row r="8" ht="78" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -983,44 +954,38 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>• Which OTP zone, and who programs it and when?</t>
+          <t>Which OTP zone? Who programs it?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>• Add 'prevent modification, replacement, deletion' (only in the verification text today).
-• Name the zone.</t>
+          <t>Add 'no modification'.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>• OTP is write-once: the overwrite test destroys a sample.
-• Test samples need a test root key.</t>
+          <t>Write-once: overwrite test destroys a sample.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>• Concept says OTP, SRS 108143 says 'protected non-volatile storage'.
-• Check free OTP size.</t>
+          <t>OTP vs 'protected NV storage' (SRS).</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>• Technical requirement copies the concept text.</t>
+          <t>TCR copies the text.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106562.
-• SRS 108143, 108142, 108144.
-• Secure-boot key (SRS 23.4) is a separate root.</t>
+          <t>MVC-106562. SRS 108143.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Lauterbach: read OTP zone; SHA-256(key) = Samsung fingerprint
-Try to write the zone -&gt; rejected; power cycle -&gt; unchanged
-SIM signs with test root -&gt; auth passes; other key -&gt; fails</t>
+          <t>Lauterbach: read OTP, compare hash
+Try write -&gt; rejected</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1052,43 +1017,38 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>• 3 retries (4 requests) or 3 attempts (3 requests)?
-• Timeout per attempt?</t>
+          <t>3 retries or 3 attempts? Timeout?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>• Request count cannot be tested without one number.
-• Define N attempts in total and timeout T.</t>
+          <t>One number needed.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>• Count requests with Saleae; SIM withholds the answer.
-• Timing untestable until T is defined.</t>
+          <t>Count requests with Saleae.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>• 'Not received' vs invalid data: is a bad signature retried?</t>
+          <t>Bad signature: retry or reject?</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>• Retry rule is split over 103053 and 103051 with different wording.</t>
+          <t>Split with 103051.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106566.
-• SRS 108124, 108126.</t>
+          <t>MVC-106566.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>SIM: no answer to the auth read; reset
-Saleae: count auth requests until SOW2 stops = N
-SIM answers on request 2 -&gt; authentication continues</t>
+          <t>SIM silent -&gt; Saleae counts requests
+SIM answers on 2nd -&gt; continues</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1120,19 +1080,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>• What is the 'expected response', and the timeout per try?
-• Same block or new SSK on retry?</t>
+          <t>What is the 'expected response'? Timeout?</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>• Define the response, the timeout and what is resent.</t>
+          <t>Define response and timeout.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>• Count with Saleae; SIM withholds the response.
-• Blocked until the response is defined.</t>
+          <t>Blocked until response is defined.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1147,15 +1105,13 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106567.
-• SRS 108149.</t>
+          <t>MVC-106567.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>SIM accepts auth, ignores the key block
-Saleae: key writes = 1 + 3 (as decided)
-SIM answers on the 2nd -&gt; session established</t>
+          <t>SIM ignores key block -&gt; Saleae counts writes
+SIM answers on 2nd -&gt; session up</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1166,7 +1122,7 @@
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
     </row>
-    <row r="11" ht="78" customHeight="1">
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1187,43 +1143,38 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>• Session lifetime?
-• Which events are a 'security failure'?
-• Reset vs restart?</t>
+          <t>Session lifetime? What is a 'security failure'?</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>• 2 of 5 triggers are untestable; conflicts with 'reject one frame and continue'.
-• Define lifetime and failure threshold; merge reset and restart.</t>
+          <t>2 of 5 triggers untestable.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>• Each trigger is testable alone; SIM replays the old key afterwards.</t>
+          <t>Each trigger testable alone.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>• Video interruption during renegotiation is not limited.</t>
+          <t>Video gap during renegotiation not limited.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>• Five triggers in one requirement: test each separately.</t>
+          <t>Five triggers in one requirement.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106573.
-• SRS 108156, 108158, 108151.</t>
+          <t>MVC-106573.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>For each trigger (expiry, reset, restart, termination, failure): establish session, fire trigger
-Saleae: new auth + new key block; SIM: SSK_new != SSK_old
-Frames with SSK_old -&gt; rejected</t>
+          <t>Per trigger: new auth + new key (Saleae)
+Old-key frames -&gt; rejected</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1234,7 +1185,7 @@
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
     </row>
-    <row r="12" ht="78" customHeight="1">
+    <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -1255,24 +1206,22 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>• Counter wrap and first-frame value after a new session?</t>
+          <t>Counter wrap and first-frame value?</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>• More than 3 lost frames blocks every later valid frame until a new session.
-• Define a recovery.</t>
+          <t>More than 3 lost frames freezes video. Add recovery.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>• Boundaries are easy (=, &lt;, +1 to +4).
-• Wrap and first frame untestable until defined.</t>
+          <t>Boundaries easy; wrap undefined.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>• Update LastAcceptedCounter only after the CMAC passes: state the order.</t>
+          <t>Update counter only after CMAC passes.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1282,16 +1231,13 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-113727.
-• SRS 108099, 108104, 108102.
-• Recovery is in no requirement.</t>
+          <t>MVC-113727. Recovery missing.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>SIM (valid CMAC): n; n again -&gt; reject; n-1 -&gt; reject; n+1, n+3 -&gt; accept; n+4 -&gt; reject
-Forged high counter + wrong tag -&gt; rejected, LastAccepted unchanged (Lauterbach)
-Skip 5 frames -&gt; observe recovery</t>
+          <t>SIM: n+1, n+3 accepted; duplicate, n+4 rejected
+Forged counter -&gt; rejected</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1302,7 +1248,7 @@
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
     </row>
-    <row r="13" ht="54" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
@@ -1323,42 +1269,38 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>• What does 'reject' do: drop, repeat previous frame, flag?</t>
+          <t>What does 'reject' do?</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>• Reaction undefined on a display camera.
-• Define: drop, count, log, continue (SRS 108105).</t>
+          <t>Define reaction: drop, log, continue.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>• Same observable as 119709: define log or counter.</t>
+          <t>Same observable as 119709.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>• No threshold for repeated bad frames.
-• Random corruption and forgery get the same reaction?</t>
+          <t>No limit for repeated bad frames.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>• Overlaps 119709 and SRS 108116.</t>
+          <t>Overlaps 119709.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106564 (ok).
-• SRS 108116, 108108, 108105.</t>
+          <t>MVC-106564.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>SIM: 10 good, 1 bad tag, 10 good
-Wireshark: bad frame missing from RTP
-Lauterbach: drop counter = 1</t>
+          <t>SIM sends 1 bad frame
+Wireshark: frame missing; log entry</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1369,7 +1311,7 @@
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n"/>
     </row>
-    <row r="14" ht="54" customHeight="1">
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1390,42 +1332,38 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>• Which commands are 'control commands'?
-• Which I2C writes are allowed before authentication?</t>
+          <t>Which commands are 'control commands'?</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>• Read literally, it forbids the writes needed to start the camera.
-• Use 'protected' and list the commands.</t>
+          <t>Literally blocks camera startup writes. List them.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>• Saleae lists all writes; the pass criterion needs the command list.</t>
+          <t>Needs the command list.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>• Volvo spec has no protected command channel.</t>
+          <t>Not in the Volvo spec.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>• Concept says 'control commands', technical says 'protected'.</t>
+          <t>'Control' vs 'protected'.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-109119.
-• SRS 108169.</t>
+          <t>MVC-109119.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Reset, auth blocked; trigger a protected command
-Saleae: only allowed pre-auth writes, no protected command
-After auth + session -&gt; command is sent</t>
+          <t>Auth blocked -&gt; Saleae: no protected writes
+Auth OK -&gt; command sent</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1436,7 +1374,7 @@
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
     </row>
-    <row r="15" ht="66" customHeight="1">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
@@ -1458,37 +1396,33 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>• 'Any accessible interface' needs a list: UART, JTAG, logs, SOME/IP/DTLS diagnostics, dumps, I2C, flash.</t>
+          <t>List the 'accessible interfaces'.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>• Negative test: needs the interface list and the SSK (from SIM).</t>
+          <t>Negative test; needs SSK from SIM.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>• SSK is in DRAM; authorised debug can read it.
-• Exclude the key region or accept an exception.</t>
+          <t>Authorised debug can read SSK in DRAM.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>• Technical requirement copies the text; SRS has 4 related requirements.</t>
+          <t>TCR copies the text.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106571.
-• SRS 108164, 108163, 108154, 108157; debug and DRAM requirements.</t>
+          <t>MVC-106571.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>SIM: get SSK; JTAG locked -&gt; Lauterbach denied
-Search I2C, Ethernet, UART captures for SSK bytes -&gt; none
-Trigger failures, read logs -&gt; no key
-Unlocked debug: read DRAM key region -&gt; record</t>
+          <t>Search all captures for SSK bytes
+JTAG locked -&gt; denied</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1520,23 +1454,22 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>• What happens to 'untrusted' video: dropped or passed with a flag? (safety decision)</t>
+          <t>'Untrusted' video: drop or flag?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>• Two very different implementations are possible.
-• Define the reaction and who evaluates it.</t>
+          <t>Define the reaction.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>• Observable only on the outgoing RTP stream or a status signal.</t>
+          <t>Observe the outgoing RTP stream.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>• 'Session established' is not defined (see 103034).</t>
+          <t>'Session established' undefined.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1546,16 +1479,13 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-109120.
-• SRS 108138.
-• Reaction is in no requirement.</t>
+          <t>MVC-109120.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Reset; SIM silent on authentication
-SIM sends frames -&gt; Wireshark: no trusted video
-Repeat after auth failure and after session end; after auth + session -&gt; video flows</t>
+          <t>Auth blocked -&gt; Wireshark: no trusted video
+Auth OK -&gt; video flows</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1566,7 +1496,7 @@
       <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n"/>
     </row>
-    <row r="17" ht="66" customHeight="1">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -1587,44 +1517,38 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>• Counter width, start value, max behaviour?
-• Does the imager check it?</t>
+          <t>Counter width, start, wrap? Imager checks it?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>• 'Monotonic' allows equal values: use 'strictly increasing, no reuse in a session' (SRS 108161).
-• State the wrap rule.</t>
+          <t>Use 'strictly increasing'.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>• Read counters with Saleae.
-• Max case needs a preset hook.</t>
+          <t>Read counters with Saleae.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>• Replay protection exists only if the imager rejects old counters.</t>
+          <t>Useless if imager ignores the counter.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>• See 113701.</t>
+          <t>See 113701.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-109121.
-• SRS 108159, 108161.</t>
+          <t>MVC-109121.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Send 100 commands; Saleae: strictly increasing
-Reset -&gt; counter restarts as defined
-Lauterbach: preset near max -&gt; new session before wrap
-If imager checks: replay old command -&gt; rejected</t>
+          <t>100 commands -&gt; counters strictly increase
+Replay old command -&gt; rejected</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1657,13 +1581,12 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>• 'New key every session' is only in the verification text: add it (SRS 108110).</t>
+          <t>Add 'new key every session'.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>• SSK is visible only through the SIM.
-• Randomness cannot be proven, only repeats.</t>
+          <t>SSK visible only via SIM.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1673,21 +1596,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>• Overlaps 103042 (how) and 103036 (new each session).
-• Keep length + new-each-session here.</t>
+          <t>Overlaps 103042 and 103036.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106568.
-• SRS 108107, 108110.</t>
+          <t>MVC-106568.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Loop 1000: reset, authenticate, SIM decrypts key block, store SSK
-Check: 32 bytes, no duplicates
-Auth failure -&gt; no key block on I2C</t>
+          <t>1000 sessions via SIM -&gt; 32 bytes, no repeats</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1698,7 +1617,7 @@
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="66" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
@@ -1719,41 +1638,38 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>• Counter width, start value, wrap, reset per stream?</t>
+          <t>Counter width, wrap, start value?</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>• Window rule cannot be checked at wrap without the width.</t>
+          <t>Width needed for the window rule.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>• Read the counter with Lauterbach.
-• SIM sends boundary values.</t>
+          <t>Read with Lauterbach.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>• Counter is protected only if the header row is inside the CMAC rows (start row 0).</t>
+          <t>Protected only if header row is in CMAC.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>• 'Use for freshness' duplicates 113703 / MVC-106575: keep extraction only.</t>
+          <t>'Use' duplicates 113703.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-113726 and MVC-106575.
-• SRS 108099.</t>
+          <t>MVC-113726, 106575.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>SIM: counters 1..N
-Lauterbach: extracted counter = sent value
-SIM: counter at max, then 0 -&gt; defined wrap; missing header -&gt; rejected</t>
+          <t>SIM counters 1..N -&gt; Lauterbach matches
+Missing header -&gt; rejected</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1764,7 +1680,7 @@
       <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
     </row>
-    <row r="20" ht="42" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
@@ -1785,41 +1701,39 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>• Footer position, length, byte order? (Samsung note missing)</t>
+          <t>Footer layout and byte order?</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>• Layout needed to implement and test.
-• Add the layout reference to the technical requirement.</t>
+          <t>Layout needed to implement and test.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>• Internal step: read the buffer with Lauterbach or infer from acceptance.</t>
+          <t>Read buffer with Lauterbach.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>• Footer is absent in frames 1-17.</t>
+          <t>No footer in frames 1-17.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>• Implementation step of 119709: keep at technical level or merge.</t>
+          <t>Step of 119709.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106572.
-• SRS 108140, 108129, 108134, 108132.</t>
+          <t>MVC-106572.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>SIM: frame with known tag T
-Lauterbach: extracted tag = T (10 different tags)
-SIM: missing or short footer -&gt; rejected, no crash</t>
+          <t>SIM sends known tag T
+Lauterbach: extracted = T
+Short footer -&gt; rejected</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1830,7 +1744,7 @@
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
     </row>
-    <row r="21" ht="78" customHeight="1">
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
@@ -1851,43 +1765,38 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>• Message layout (SSK, Row_info_00/01), OAEP label, MGF1 hash? (Samsung note missing)</t>
+          <t>Message layout, OAEP label, MGF1?</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>• Layout is needed by implementation and test: put it in the technical requirement.</t>
+          <t>Put layout in the technical requirement.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>• OAEP is randomised: compare plaintexts only.
-• Known SSK needs a test hook.</t>
+          <t>OAEP is random: compare plaintext only.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>• RSA-2048 OAEP/SHA-256 holds max 190 bytes: 32-byte SSK + Row_info fits.
-• Row rules depend on the output mode.</t>
+          <t>OAEP limit 190 bytes: SSK + Row_info fits.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>• 4 technical requirements, 3 about row selection: give row selection its own concept requirement.</t>
+          <t>Row rules need own requirement.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106580, 106576, 108741, 106574.
-• SRS 108153, 108145, 108165, 108166.</t>
+          <t>MVC-106580, 106576, 108741, 106574.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>SIM: decrypt key block (OAEP, SHA-256) -&gt; SSK + Row_info
-Lauterbach: Row_info used = decrypted
-Wrong private key -&gt; fails; no SSK in plaintext on I2C
-Bad row settings -&gt; refused</t>
+          <t>SIM decrypts key block -&gt; SSK + Row_info
+Wrong key -&gt; fails</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1919,43 +1828,38 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>• Exact CMAC input bytes: pixel data only, or line headers too?
-• Row numbering base?</t>
+          <t>Exact CMAC input bytes?</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>• Two implementations could produce different tags.
-• Add exact input and a Samsung test vector.</t>
+          <t>Add exact input + test vector.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>• Reference calculation needs the SSK and exact input: SIM only.</t>
+          <t>Needs SSK: SIM only.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>• AES-256 CMAC, full 128-bit tag: state 'not truncated'.
-• No host-side speed requirement.</t>
+          <t>State full 128-bit tag.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>• Row selection is defined in 4 other requirements: give it its own concept requirement.</t>
+          <t>Row selection needs own requirement.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106583.
-• SRS 108122, 108121, 108118.</t>
+          <t>MVC-106583.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>TE-1190: capture frame rows
-PyRef: tag = AES256-CMAC(SSK, selected rows)
-SIM: send -&gt; accepted; change 1 byte in a selected row -&gt; rejected; in an unselected row -&gt; accepted</t>
+          <t>PyRef tag -&gt; SIM sends -&gt; accepted
+Change selected byte -&gt; rejected</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1966,7 +1870,7 @@
       <c r="M22" s="2" t="n"/>
       <c r="N22" s="2" t="n"/>
     </row>
-    <row r="23" ht="54" customHeight="1">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
@@ -1987,44 +1891,38 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>• Does the imager verify command tags at all?
-• Command format and CMAC input?</t>
+          <t>Does the imager check command tags?</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>• If the imager does not check, the tag adds nothing: confirm first.
-• Then fix the input (command + counter, SRS 108159).</t>
+          <t>Confirm support; fix CMAC input.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>• Tag checkable with PyRef.
-• Imager rejection untestable if it does not check.</t>
+          <t>Imager rejection untestable if unchecked.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>• Concept: 'each command'. SRS: 'only when supported by SOW1'. Conflict.</t>
+          <t>Concept 'each'; SRS 'only if supported'.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>• 113701, 119707, 113702 are steps of one function: merge into one 'protected command format'.</t>
+          <t>Merge with 119707, 113702.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-108740.
-• SRS 108160, 108159.</t>
+          <t>MVC-108740.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Trigger a protected command
-Saleae: parse cmd | counter | tag
-PyRef: AES256-CMAC(SSK, cmd||counter) = tag
-If imager checks: wrong tag -&gt; rejected</t>
+          <t>Saleae: parse cmd | counter | tag
+PyRef recomputes tag -&gt; equal</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2035,7 +1933,7 @@
       <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
     </row>
-    <row r="24" ht="78" customHeight="1">
+    <row r="24" ht="66" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
@@ -2056,43 +1954,39 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>• Define Device_n, KID, Sig_device and the exact signed message (Volvo spec: key + Device ID).</t>
+          <t>Define Device_n, KID, signed message.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>• Signed message must be defined byte for byte, or SOW2 and test disagree.</t>
+          <t>Signed data must be byte-exact.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>• Needs signatures from a test root key.
-• Negative cases need the SIM.</t>
+          <t>Needs test root key + SIM.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>• Signature is static (no challenge): a copied record passes this step.
-• Only the CMAC (frame 18+) proves the private key.
-• Concept fixes the scheme, SRS lets KID choose.</t>
+          <t>Static signature: a copied record passes.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>• Three technical requirements verify it: keep tests separate per topic.</t>
+          <t>Three technical requirements verify it.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106561/106565/106563.
-• SRS 108133, 108131, 108126, 108124, 108113, 108111.</t>
+          <t>MVC-106561, 106565, 106563.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>SIM serves genuine data -&gt; Saleae: key block follows
-Flip 1 bit in Device_n / KID / Sig -&gt; rejected, no key sent
-Replay genuine data without the private key -&gt; auth passes, frames rejected</t>
+          <t>SIM genuine -&gt; key block follows
+Flip 1 bit -&gt; rejected
+Replayed copy -&gt; no valid frames</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2103,7 +1997,7 @@
       <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="n"/>
     </row>
-    <row r="25" ht="54" customHeight="1">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
@@ -2124,41 +2018,38 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>• Field order and size in the I2C write?
-• Where does the I2C CRC go?</t>
+          <t>Field order? Position of I2C CRC?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>• Define the layout in the technical requirement, with an example.</t>
+          <t>Define layout with an example.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>• Easy with Saleae once the layout is defined.</t>
+          <t>Easy with Saleae.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>• If CMAC generation fails, no command may be sent (SRS 108160): add it.</t>
+          <t>No command if CMAC fails.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>• See 113701.</t>
+          <t>See 113701.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106570.
-• SRS 108160.</t>
+          <t>MVC-106570.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Saleae: write = [cmd][counter][16-byte tag] in the defined order
-Lauterbach: force CMAC failure -&gt; nothing sent
-Repeat for 3 commands</t>
+          <t>Saleae: [cmd][counter][tag]
+Force CMAC failure -&gt; nothing sent</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2169,7 +2060,7 @@
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
     </row>
-    <row r="26" ht="66" customHeight="1">
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
@@ -2190,22 +2081,22 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>• Key format: modulus only? Fixed exponent?</t>
+          <t>Key format and exponent?</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>• Add sanity checks (2048 bit, odd modulus, exponent) before use.</t>
+          <t>Add key sanity checks.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>• Internal: check indirectly. SIM decrypts the key block with its private key.</t>
+          <t>SIM decrypt proves the right key.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>• Key is covered by the signature only if Device_n is the modulus.</t>
+          <t>Signature must cover the key.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2215,15 +2106,13 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>• Linked to MVC-106577.
-• SRS 108153.</t>
+          <t>MVC-106577.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>SIM: decrypt SOW2's key block with K1 private -&gt; success
-SIM key of 1024 or 4096 bits, valid signature -&gt; rejected
-Truncated or zero key -&gt; rejected</t>
+          <t>SIM decrypts key block -&gt; ok
+Wrong-size key -&gt; rejected</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">

</xml_diff>